<commit_message>
Se ajustaron los templates para que los pdf salieran bien
</commit_message>
<xml_diff>
--- a/backend/templates/reportes/Ficha - Practicas libres.xlsx
+++ b/backend/templates/reportes/Ficha - Practicas libres.xlsx
@@ -1,15 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F5CD89C-A9F2-4659-BA11-C498BC4EE64C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B91DDE63-73CE-4AF2-A3FC-19AAD3E53EF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28560" windowHeight="13905" xr2:uid="{A22C7B05-6B0A-4116-A99A-60EDDEA67682}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A22C7B05-6B0A-4116-A99A-60EDDEA67682}"/>
   </bookViews>
   <sheets>
     <sheet name="Ficha - PracticasLibres" sheetId="2" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Ficha - PracticasLibres'!$A$1:$L$31</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -44,7 +47,7 @@
         <b/>
         <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -54,7 +57,7 @@
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -67,7 +70,7 @@
         <b/>
         <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -77,7 +80,7 @@
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -90,7 +93,7 @@
         <b/>
         <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -100,7 +103,7 @@
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -113,7 +116,7 @@
         <b/>
         <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -123,7 +126,7 @@
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -136,7 +139,7 @@
         <b/>
         <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -146,7 +149,7 @@
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -162,7 +165,7 @@
         <u/>
         <sz val="10"/>
         <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -172,7 +175,7 @@
       <rPr>
         <sz val="10"/>
         <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -249,7 +252,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -260,14 +263,14 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -275,7 +278,7 @@
       <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -283,14 +286,14 @@
       <u/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -298,7 +301,7 @@
       <b/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -306,7 +309,7 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -526,6 +529,105 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -537,105 +639,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -754,9 +757,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -794,7 +797,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -900,7 +903,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1042,7 +1045,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1054,7 +1057,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1:S32"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" customHeight="1" zeroHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="8.140625" style="1" customWidth="1"/>
@@ -1073,157 +1076,157 @@
     <col min="19" max="16384" width="9.140625" style="8" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:19" ht="15.75" customHeight="1">
+    <row r="1" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="O1"/>
       <c r="P1"/>
       <c r="Q1"/>
       <c r="R1"/>
       <c r="S1"/>
     </row>
-    <row r="2" spans="2:19" ht="15" customHeight="1">
-      <c r="B2" s="35"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="41" t="s">
+    <row r="2" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="12"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="27"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="45" t="s">
+      <c r="E2" s="19"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="42"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="36"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="13"/>
       <c r="O2"/>
       <c r="P2"/>
       <c r="Q2"/>
       <c r="R2"/>
       <c r="S2"/>
     </row>
-    <row r="3" spans="2:19" ht="15.75" customHeight="1">
-      <c r="B3" s="37"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="44"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="38"/>
+    <row r="3" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="14"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="26"/>
+      <c r="K3" s="15"/>
       <c r="O3"/>
       <c r="P3"/>
       <c r="Q3"/>
       <c r="R3"/>
       <c r="S3"/>
     </row>
-    <row r="4" spans="2:19" ht="15" customHeight="1">
-      <c r="B4" s="37"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="45" t="s">
+    <row r="4" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="14"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="27"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="45" t="s">
+      <c r="E4" s="19"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="42"/>
-      <c r="I4" s="37"/>
-      <c r="J4" s="47"/>
-      <c r="K4" s="38"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="15"/>
       <c r="O4"/>
       <c r="P4"/>
       <c r="Q4"/>
       <c r="R4"/>
       <c r="S4"/>
     </row>
-    <row r="5" spans="2:19" ht="15.75" customHeight="1">
-      <c r="B5" s="37"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="37"/>
-      <c r="J5" s="47"/>
-      <c r="K5" s="38"/>
+    <row r="5" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="14"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="26"/>
+      <c r="K5" s="15"/>
       <c r="O5"/>
       <c r="P5"/>
       <c r="Q5"/>
       <c r="R5"/>
       <c r="S5"/>
     </row>
-    <row r="6" spans="2:19" ht="15" customHeight="1">
-      <c r="B6" s="37"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="45" t="s">
+    <row r="6" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="14"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="27"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="45" t="s">
+      <c r="E6" s="19"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="42"/>
-      <c r="I6" s="37"/>
-      <c r="J6" s="47"/>
-      <c r="K6" s="38"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="15"/>
       <c r="O6"/>
       <c r="P6"/>
       <c r="Q6"/>
       <c r="R6"/>
       <c r="S6"/>
     </row>
-    <row r="7" spans="2:19" ht="15.75" customHeight="1">
-      <c r="B7" s="39"/>
-      <c r="C7" s="40"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="44"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="44"/>
-      <c r="I7" s="39"/>
-      <c r="J7" s="48"/>
-      <c r="K7" s="40"/>
+    <row r="7" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="16"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="27"/>
+      <c r="K7" s="17"/>
       <c r="O7"/>
       <c r="P7"/>
       <c r="Q7"/>
       <c r="R7"/>
       <c r="S7"/>
     </row>
-    <row r="8" spans="2:19" ht="15" customHeight="1">
-      <c r="B8" s="27" t="s">
+    <row r="8" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="27"/>
-      <c r="K8" s="27"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
       <c r="O8"/>
       <c r="P8"/>
       <c r="Q8"/>
       <c r="R8"/>
       <c r="S8"/>
     </row>
-    <row r="9" spans="2:19">
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
-      <c r="K9" s="28"/>
+    <row r="9" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
       <c r="O9"/>
       <c r="P9"/>
       <c r="Q9"/>
@@ -1232,59 +1235,59 @@
       </c>
       <c r="S9"/>
     </row>
-    <row r="10" spans="2:19" ht="15" customHeight="1">
-      <c r="B10" s="29" t="s">
+    <row r="10" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="29" t="s">
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="H10" s="30"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="30"/>
-      <c r="K10" s="31"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
+      <c r="K10" s="30"/>
       <c r="O10"/>
       <c r="P10"/>
       <c r="Q10"/>
       <c r="R10"/>
       <c r="S10"/>
     </row>
-    <row r="11" spans="2:19" ht="15.75" customHeight="1">
-      <c r="B11" s="32"/>
-      <c r="C11" s="33"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="33"/>
-      <c r="I11" s="33"/>
-      <c r="J11" s="33"/>
-      <c r="K11" s="34"/>
+    <row r="11" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="31"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="32"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="33"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="32"/>
+      <c r="K11" s="33"/>
       <c r="O11"/>
       <c r="P11"/>
       <c r="Q11"/>
       <c r="R11"/>
       <c r="S11"/>
     </row>
-    <row r="12" spans="2:19" ht="15" customHeight="1">
-      <c r="B12" s="29" t="s">
+    <row r="12" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="31"/>
-      <c r="G12" s="29" t="s">
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="H12" s="30"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="30"/>
-      <c r="K12" s="31"/>
+      <c r="H12" s="29"/>
+      <c r="I12" s="29"/>
+      <c r="J12" s="29"/>
+      <c r="K12" s="30"/>
       <c r="O12"/>
       <c r="P12"/>
       <c r="Q12"/>
@@ -1293,24 +1296,24 @@
       </c>
       <c r="S12"/>
     </row>
-    <row r="13" spans="2:19">
-      <c r="B13" s="32"/>
-      <c r="C13" s="33"/>
-      <c r="D13" s="33"/>
-      <c r="E13" s="33"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="33"/>
-      <c r="I13" s="33"/>
-      <c r="J13" s="33"/>
-      <c r="K13" s="34"/>
+    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B13" s="31"/>
+      <c r="C13" s="32"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="33"/>
       <c r="O13"/>
       <c r="P13"/>
       <c r="Q13"/>
       <c r="R13"/>
       <c r="S13"/>
     </row>
-    <row r="14" spans="2:19" ht="6.75" customHeight="1">
+    <row r="14" spans="2:19" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -1327,7 +1330,7 @@
       <c r="R14"/>
       <c r="S14"/>
     </row>
-    <row r="15" spans="2:19">
+    <row r="15" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
         <v>12</v>
       </c>
@@ -1358,24 +1361,24 @@
       </c>
       <c r="S15"/>
     </row>
-    <row r="16" spans="2:19" ht="15.75" customHeight="1">
+    <row r="16" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="16"/>
-      <c r="J16" s="17"/>
-      <c r="K16" s="18"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="35"/>
+      <c r="H16" s="36"/>
+      <c r="I16" s="34"/>
+      <c r="J16" s="35"/>
+      <c r="K16" s="36"/>
       <c r="O16"/>
       <c r="P16"/>
       <c r="Q16"/>
       <c r="R16"/>
       <c r="S16"/>
     </row>
-    <row r="17" spans="2:19" ht="6.75" customHeight="1">
+    <row r="17" spans="2:19" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -1392,18 +1395,18 @@
       <c r="R17"/>
       <c r="S17"/>
     </row>
-    <row r="18" spans="2:19">
-      <c r="B18" s="19" t="s">
+    <row r="18" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B18" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="19" t="s">
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="41"/>
+      <c r="H18" s="37" t="s">
         <v>21</v>
       </c>
       <c r="I18" s="9" t="s">
@@ -1419,14 +1422,14 @@
       </c>
       <c r="S18"/>
     </row>
-    <row r="19" spans="2:19">
-      <c r="B19" s="20"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="20"/>
+    <row r="19" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B19" s="38"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="43"/>
+      <c r="F19" s="43"/>
+      <c r="G19" s="44"/>
+      <c r="H19" s="38"/>
       <c r="I19" s="4" t="s">
         <v>24</v>
       </c>
@@ -1442,7 +1445,7 @@
       </c>
       <c r="S19"/>
     </row>
-    <row r="20" spans="2:19" ht="15.75" customHeight="1">
+    <row r="20" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="4"/>
       <c r="C20" s="9"/>
       <c r="D20" s="10"/>
@@ -1459,7 +1462,7 @@
       <c r="R20"/>
       <c r="S20"/>
     </row>
-    <row r="21" spans="2:19" ht="15.75" customHeight="1">
+    <row r="21" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="4"/>
       <c r="C21" s="9"/>
       <c r="D21" s="10"/>
@@ -1476,7 +1479,7 @@
       <c r="R21"/>
       <c r="S21"/>
     </row>
-    <row r="22" spans="2:19" ht="15.75" customHeight="1">
+    <row r="22" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="4"/>
       <c r="C22" s="9"/>
       <c r="D22" s="10"/>
@@ -1493,7 +1496,7 @@
       <c r="R22"/>
       <c r="S22"/>
     </row>
-    <row r="23" spans="2:19" ht="15.75" customHeight="1">
+    <row r="23" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="4"/>
       <c r="C23" s="9"/>
       <c r="D23" s="10"/>
@@ -1510,7 +1513,7 @@
       <c r="R23"/>
       <c r="S23"/>
     </row>
-    <row r="24" spans="2:19">
+    <row r="24" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
@@ -1527,105 +1530,105 @@
       <c r="R24"/>
       <c r="S24"/>
     </row>
-    <row r="25" spans="2:19" ht="44.25" customHeight="1">
-      <c r="B25" s="12" t="s">
+    <row r="25" spans="2:19" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="12"/>
-      <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
+      <c r="C25" s="45"/>
+      <c r="D25" s="45"/>
+      <c r="E25" s="45"/>
+      <c r="F25" s="45"/>
+      <c r="G25" s="45"/>
+      <c r="H25" s="45"/>
+      <c r="I25" s="45"/>
+      <c r="J25" s="45"/>
+      <c r="K25" s="45"/>
       <c r="O25"/>
       <c r="P25"/>
       <c r="Q25"/>
       <c r="R25"/>
       <c r="S25"/>
     </row>
-    <row r="26" spans="2:19">
-      <c r="B26" s="13" t="s">
+    <row r="26" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B26" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="14" t="str">
+      <c r="C26" s="46"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="46"/>
+      <c r="G26" s="47" t="str">
         <f>SUBSTITUTE("USUARIO: " &amp; B10,"NOMBRE:","")</f>
         <v xml:space="preserve">USUARIO: </v>
       </c>
-      <c r="H26" s="14"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
+      <c r="H26" s="47"/>
+      <c r="I26" s="47"/>
+      <c r="J26" s="47"/>
+      <c r="K26" s="47"/>
       <c r="O26"/>
       <c r="P26"/>
       <c r="Q26"/>
       <c r="R26"/>
       <c r="S26"/>
     </row>
-    <row r="27" spans="2:19">
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="14"/>
-      <c r="J27" s="14"/>
-      <c r="K27" s="14"/>
+    <row r="27" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B27" s="46"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="47"/>
+      <c r="H27" s="47"/>
+      <c r="I27" s="47"/>
+      <c r="J27" s="47"/>
+      <c r="K27" s="47"/>
       <c r="O27"/>
       <c r="P27"/>
       <c r="Q27"/>
       <c r="R27"/>
       <c r="S27"/>
     </row>
-    <row r="28" spans="2:19">
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="15" t="s">
+    <row r="28" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B28" s="46"/>
+      <c r="C28" s="46"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="46"/>
+      <c r="G28" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="H28" s="15"/>
-      <c r="I28" s="15"/>
-      <c r="J28" s="15"/>
-      <c r="K28" s="15"/>
+      <c r="H28" s="48"/>
+      <c r="I28" s="48"/>
+      <c r="J28" s="48"/>
+      <c r="K28" s="48"/>
       <c r="O28"/>
       <c r="P28"/>
       <c r="Q28"/>
       <c r="R28"/>
       <c r="S28"/>
     </row>
-    <row r="29" spans="2:19">
+    <row r="29" spans="2:19" x14ac:dyDescent="0.25">
       <c r="O29"/>
       <c r="P29"/>
       <c r="Q29"/>
       <c r="R29"/>
       <c r="S29"/>
     </row>
-    <row r="30" spans="2:19">
+    <row r="30" spans="2:19" x14ac:dyDescent="0.25">
       <c r="O30"/>
       <c r="P30"/>
       <c r="Q30"/>
       <c r="R30"/>
       <c r="S30"/>
     </row>
-    <row r="31" spans="2:19">
+    <row r="31" spans="2:19" x14ac:dyDescent="0.25">
       <c r="O31"/>
       <c r="P31"/>
       <c r="Q31"/>
       <c r="R31"/>
       <c r="S31"/>
     </row>
-    <row r="32" spans="2:19" ht="15" hidden="1" customHeight="1">
+    <row r="32" spans="2:19" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="O32"/>
       <c r="P32"/>
       <c r="Q32"/>
@@ -1634,6 +1637,25 @@
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="B25:K25"/>
+    <mergeCell ref="B26:F28"/>
+    <mergeCell ref="G26:K27"/>
+    <mergeCell ref="G28:K28"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:G19"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="J19:K19"/>
     <mergeCell ref="F15:H15"/>
     <mergeCell ref="I15:K15"/>
     <mergeCell ref="B2:C7"/>
@@ -1649,28 +1671,10 @@
     <mergeCell ref="G10:K11"/>
     <mergeCell ref="B12:F13"/>
     <mergeCell ref="G12:K13"/>
-    <mergeCell ref="F16:H16"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:G19"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="C20:G20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="B25:K25"/>
-    <mergeCell ref="B26:F28"/>
-    <mergeCell ref="G26:K27"/>
-    <mergeCell ref="G28:K28"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.23622047244094491" right="0.74803149606299213" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="110" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>